<commit_message>
update provider costs files
</commit_message>
<xml_diff>
--- a/provider_specialty_cprd_V.0.1.xlsx
+++ b/provider_specialty_cprd_V.0.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioxfordnexus-my.sharepoint.com/personal/orms1149_ox_ac_uk/Documents/Documents/GitHub/OMOP-Validation-Study/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{89A282C8-6E18-42A4-9AD7-5AC0F61BDD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F9892AB-2575-4618-8E24-12F160490F4E}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{89A282C8-6E18-42A4-9AD7-5AC0F61BDD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8A0A917-C64C-4DF4-8AE0-942DAA805261}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{2735BDA3-DE0F-409A-AF31-62DE8638BF76}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2735BDA3-DE0F-409A-AF31-62DE8638BF76}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -706,15 +706,14 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{C93FE370-54C2-4E7D-B78B-D5F64D6ECB73}"/>
@@ -1074,10 +1073,10 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="2">
@@ -1085,10 +1084,10 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="1">
         <v>1</v>
       </c>
       <c r="C3" s="2">
@@ -1096,10 +1095,10 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="1">
         <v>1</v>
       </c>
       <c r="C4" s="2">
@@ -1158,10 +1157,10 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="1">
         <v>1</v>
       </c>
       <c r="C11" s="2">
@@ -1223,10 +1222,10 @@
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="1">
         <v>1</v>
       </c>
       <c r="C18" s="2">
@@ -1234,10 +1233,10 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="5">
+      <c r="B19" s="1">
         <v>1</v>
       </c>
       <c r="C19" s="2">
@@ -1253,10 +1252,10 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="1">
         <v>1</v>
       </c>
       <c r="C21" s="2">
@@ -1280,10 +1279,10 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="5">
+      <c r="B24" s="1">
         <v>1</v>
       </c>
       <c r="C24" s="2">
@@ -1348,10 +1347,10 @@
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="5">
+      <c r="B31" s="1">
         <v>1</v>
       </c>
       <c r="C31" s="2">
@@ -1367,10 +1366,10 @@
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B33" s="5">
+      <c r="B33" s="1">
         <v>1</v>
       </c>
       <c r="C33" s="2">
@@ -1426,10 +1425,10 @@
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B40" s="5">
+      <c r="B40" s="1">
         <v>1</v>
       </c>
       <c r="C40" s="2">
@@ -1453,10 +1452,10 @@
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B43" s="5">
+      <c r="B43" s="1">
         <v>1</v>
       </c>
       <c r="C43" s="2">
@@ -1464,13 +1463,13 @@
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B44" s="5">
-        <v>1</v>
-      </c>
-      <c r="C44" s="5">
+      <c r="B44" s="1">
+        <v>1</v>
+      </c>
+      <c r="C44" s="1">
         <v>28.5</v>
       </c>
     </row>
@@ -1483,21 +1482,21 @@
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B46" s="5">
-        <v>1</v>
-      </c>
-      <c r="C46" s="5">
+      <c r="B46" s="1">
+        <v>1</v>
+      </c>
+      <c r="C46" s="1">
         <v>6.2</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="5" t="s">
+      <c r="A47" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B47" s="5">
+      <c r="B47" s="1">
         <v>1</v>
       </c>
       <c r="C47" s="2">
@@ -1513,13 +1512,13 @@
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="5" t="s">
+      <c r="A49" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B49" s="5">
-        <v>1</v>
-      </c>
-      <c r="C49" s="5">
+      <c r="B49" s="1">
+        <v>1</v>
+      </c>
+      <c r="C49" s="1">
         <v>23</v>
       </c>
     </row>
@@ -1559,10 +1558,10 @@
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="5" t="s">
+      <c r="A54" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B54" s="5">
+      <c r="B54" s="1">
         <v>1</v>
       </c>
       <c r="C54" s="2">
@@ -1570,10 +1569,10 @@
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="5" t="s">
+      <c r="A55" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B55" s="5">
+      <c r="B55" s="1">
         <v>1</v>
       </c>
       <c r="C55" s="2">
@@ -1581,10 +1580,10 @@
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="5" t="s">
+      <c r="A56" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B56" s="5">
+      <c r="B56" s="1">
         <v>1</v>
       </c>
       <c r="C56" s="2">
@@ -1592,10 +1591,10 @@
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="5" t="s">
+      <c r="A57" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B57" s="5">
+      <c r="B57" s="1">
         <v>1</v>
       </c>
       <c r="C57" s="2">
@@ -1611,10 +1610,10 @@
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="5" t="s">
+      <c r="A59" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B59" s="5">
+      <c r="B59" s="1">
         <v>1</v>
       </c>
       <c r="C59" s="2">
@@ -1646,10 +1645,10 @@
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="5" t="s">
+      <c r="A63" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B63" s="5">
+      <c r="B63" s="1">
         <v>1</v>
       </c>
       <c r="C63" s="2">
@@ -1657,10 +1656,10 @@
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="5" t="s">
+      <c r="A64" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B64" s="5">
+      <c r="B64" s="1">
         <v>1</v>
       </c>
       <c r="C64" s="2">
@@ -1668,10 +1667,10 @@
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="5" t="s">
+      <c r="A65" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B65" s="5">
+      <c r="B65" s="1">
         <v>1</v>
       </c>
       <c r="C65" s="2">
@@ -1716,10 +1715,10 @@
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="5" t="s">
+      <c r="A71" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B71" s="5">
+      <c r="B71" s="1">
         <v>1</v>
       </c>
       <c r="C71" s="2">
@@ -1727,10 +1726,10 @@
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="5" t="s">
+      <c r="A72" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B72" s="5">
+      <c r="B72" s="1">
         <v>1</v>
       </c>
       <c r="C72" s="2">
@@ -1738,10 +1737,10 @@
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="5" t="s">
+      <c r="A73" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B73" s="5">
+      <c r="B73" s="1">
         <v>1</v>
       </c>
       <c r="C73" s="2">
@@ -1781,10 +1780,10 @@
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A78" s="5" t="s">
+      <c r="A78" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B78" s="5">
+      <c r="B78" s="1">
         <v>1</v>
       </c>
       <c r="C78" s="2">
@@ -1808,10 +1807,10 @@
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A81" s="5" t="s">
+      <c r="A81" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B81" s="5">
+      <c r="B81" s="1">
         <v>1</v>
       </c>
       <c r="C81" s="2">
@@ -1827,10 +1826,10 @@
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A83" s="5" t="s">
+      <c r="A83" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B83" s="5">
+      <c r="B83" s="1">
         <v>1</v>
       </c>
       <c r="C83" s="2">
@@ -1838,10 +1837,10 @@
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A84" s="5" t="s">
+      <c r="A84" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B84" s="5">
+      <c r="B84" s="1">
         <v>1</v>
       </c>
       <c r="C84" s="2">
@@ -1849,21 +1848,21 @@
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A85" s="5" t="s">
+      <c r="A85" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B85" s="5">
-        <v>1</v>
-      </c>
-      <c r="C85" s="5">
+      <c r="B85" s="1">
+        <v>1</v>
+      </c>
+      <c r="C85" s="1">
         <v>11.5</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A86" s="5" t="s">
+      <c r="A86" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B86" s="5">
+      <c r="B86" s="1">
         <v>1</v>
       </c>
       <c r="C86" s="2">
@@ -1871,10 +1870,10 @@
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A87" s="5" t="s">
+      <c r="A87" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B87" s="5">
+      <c r="B87" s="1">
         <v>1</v>
       </c>
       <c r="C87" s="2">
@@ -1882,10 +1881,10 @@
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A88" s="5" t="s">
+      <c r="A88" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B88" s="5">
+      <c r="B88" s="1">
         <v>1</v>
       </c>
       <c r="C88" s="2">
@@ -1893,10 +1892,10 @@
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A89" s="5" t="s">
+      <c r="A89" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B89" s="5">
+      <c r="B89" s="1">
         <v>1</v>
       </c>
       <c r="C89" s="2">
@@ -1912,10 +1911,10 @@
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A91" s="5" t="s">
+      <c r="A91" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B91" s="5">
+      <c r="B91" s="1">
         <v>1</v>
       </c>
       <c r="C91" s="2">
@@ -1931,10 +1930,10 @@
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A93" s="5" t="s">
+      <c r="A93" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B93" s="5">
+      <c r="B93" s="1">
         <v>1</v>
       </c>
       <c r="C93" s="2">
@@ -1942,10 +1941,10 @@
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A94" s="5" t="s">
+      <c r="A94" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B94" s="5">
+      <c r="B94" s="1">
         <v>1</v>
       </c>
       <c r="C94" s="2">
@@ -1961,10 +1960,10 @@
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A96" s="5" t="s">
+      <c r="A96" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B96" s="5">
+      <c r="B96" s="1">
         <v>1</v>
       </c>
       <c r="C96" s="2">
@@ -1980,21 +1979,21 @@
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A98" s="5" t="s">
+      <c r="A98" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B98" s="5">
-        <v>1</v>
-      </c>
-      <c r="C98" s="5">
+      <c r="B98" s="1">
+        <v>1</v>
+      </c>
+      <c r="C98" s="1">
         <v>6.2</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A99" s="5" t="s">
+      <c r="A99" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B99" s="5">
+      <c r="B99" s="1">
         <v>1</v>
       </c>
       <c r="C99" s="2">
@@ -2002,21 +2001,21 @@
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A100" s="5" t="s">
+      <c r="A100" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B100" s="5">
-        <v>1</v>
-      </c>
-      <c r="C100" s="5">
+      <c r="B100" s="1">
+        <v>1</v>
+      </c>
+      <c r="C100" s="1">
         <v>26.75</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A101" s="5" t="s">
+      <c r="A101" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B101" s="5">
+      <c r="B101" s="1">
         <v>1</v>
       </c>
       <c r="C101" s="2">
@@ -2032,10 +2031,10 @@
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A103" s="5" t="s">
+      <c r="A103" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B103" s="5">
+      <c r="B103" s="1">
         <v>1</v>
       </c>
       <c r="C103" s="2">
@@ -2043,10 +2042,10 @@
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A104" s="5" t="s">
+      <c r="A104" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B104" s="5">
+      <c r="B104" s="1">
         <v>1</v>
       </c>
       <c r="C104" s="2">
@@ -2054,10 +2053,10 @@
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A105" s="5" t="s">
+      <c r="A105" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B105" s="5">
+      <c r="B105" s="1">
         <v>1</v>
       </c>
       <c r="C105" s="2">
@@ -2073,13 +2072,13 @@
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A107" s="5" t="s">
+      <c r="A107" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B107" s="5">
-        <v>1</v>
-      </c>
-      <c r="C107" s="5">
+      <c r="B107" s="1">
+        <v>1</v>
+      </c>
+      <c r="C107" s="1">
         <v>6.2</v>
       </c>
     </row>
@@ -2108,10 +2107,10 @@
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A111" s="5" t="s">
+      <c r="A111" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B111" s="5">
+      <c r="B111" s="1">
         <v>1</v>
       </c>
       <c r="C111" s="2">
@@ -2119,10 +2118,10 @@
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A112" s="5" t="s">
+      <c r="A112" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B112" s="5">
+      <c r="B112" s="1">
         <v>1</v>
       </c>
       <c r="C112" s="2">
@@ -2170,10 +2169,10 @@
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A118" s="5" t="s">
+      <c r="A118" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="B118" s="5">
+      <c r="B118" s="1">
         <v>1</v>
       </c>
       <c r="C118" s="2">
@@ -2181,10 +2180,10 @@
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A119" s="5" t="s">
+      <c r="A119" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B119" s="5">
+      <c r="B119" s="1">
         <v>1</v>
       </c>
       <c r="C119" s="2">
@@ -2192,10 +2191,10 @@
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A120" s="5" t="s">
+      <c r="A120" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B120" s="5">
+      <c r="B120" s="1">
         <v>1</v>
       </c>
       <c r="C120" s="2">
@@ -2203,10 +2202,10 @@
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A121" s="5" t="s">
+      <c r="A121" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B121" s="5">
+      <c r="B121" s="1">
         <v>1</v>
       </c>
       <c r="C121" s="2">
@@ -2222,21 +2221,21 @@
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A123" s="5" t="s">
+      <c r="A123" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B123" s="5">
-        <v>1</v>
-      </c>
-      <c r="C123" s="5">
+      <c r="B123" s="1">
+        <v>1</v>
+      </c>
+      <c r="C123" s="1">
         <v>50</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A124" s="5" t="s">
+      <c r="A124" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B124" s="5">
+      <c r="B124" s="1">
         <v>1</v>
       </c>
       <c r="C124" s="2">
@@ -2244,13 +2243,13 @@
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A125" s="5" t="s">
+      <c r="A125" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B125" s="5">
-        <v>1</v>
-      </c>
-      <c r="C125" s="5">
+      <c r="B125" s="1">
+        <v>1</v>
+      </c>
+      <c r="C125" s="1">
         <v>107.26</v>
       </c>
     </row>
@@ -2263,10 +2262,10 @@
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A127" s="5" t="s">
+      <c r="A127" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B127" s="5">
+      <c r="B127" s="1">
         <v>1</v>
       </c>
       <c r="C127" s="2">
@@ -2274,10 +2273,10 @@
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A128" s="5" t="s">
+      <c r="A128" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B128" s="5">
+      <c r="B128" s="1">
         <v>1</v>
       </c>
       <c r="C128" s="2">
@@ -2285,10 +2284,10 @@
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A129" s="5" t="s">
+      <c r="A129" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B129" s="5">
+      <c r="B129" s="1">
         <v>1</v>
       </c>
       <c r="C129" s="2">
@@ -2296,13 +2295,13 @@
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A130" s="5" t="s">
+      <c r="A130" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B130" s="5">
-        <v>1</v>
-      </c>
-      <c r="C130" s="5">
+      <c r="B130" s="1">
+        <v>1</v>
+      </c>
+      <c r="C130" s="1">
         <v>104</v>
       </c>
     </row>
@@ -2323,10 +2322,10 @@
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A133" s="5" t="s">
+      <c r="A133" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B133" s="5">
+      <c r="B133" s="1">
         <v>1</v>
       </c>
       <c r="C133" s="2">
@@ -2342,10 +2341,10 @@
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A135" s="5" t="s">
+      <c r="A135" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B135" s="5">
+      <c r="B135" s="1">
         <v>1</v>
       </c>
       <c r="C135" s="2">
@@ -2372,10 +2371,10 @@
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A138" s="5" t="s">
+      <c r="A138" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B138" s="5">
+      <c r="B138" s="1">
         <v>1</v>
       </c>
       <c r="C138" s="2">
@@ -2423,10 +2422,10 @@
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A144" s="5" t="s">
+      <c r="A144" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B144" s="5">
+      <c r="B144" s="1">
         <v>1</v>
       </c>
       <c r="C144" s="2">
@@ -2434,13 +2433,13 @@
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A145" s="5" t="s">
+      <c r="A145" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B145" s="5">
-        <v>1</v>
-      </c>
-      <c r="C145" s="5">
+      <c r="B145" s="1">
+        <v>1</v>
+      </c>
+      <c r="C145" s="1">
         <v>156.82</v>
       </c>
     </row>
@@ -2453,10 +2452,10 @@
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A147" s="5" t="s">
+      <c r="A147" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B147" s="5">
+      <c r="B147" s="1">
         <v>1</v>
       </c>
       <c r="C147" s="2">
@@ -2488,10 +2487,10 @@
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A151" s="5" t="s">
+      <c r="A151" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B151" s="5">
+      <c r="B151" s="1">
         <v>1</v>
       </c>
       <c r="C151" s="2">
@@ -2507,10 +2506,10 @@
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A153" s="5" t="s">
+      <c r="A153" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B153" s="5">
+      <c r="B153" s="1">
         <v>1</v>
       </c>
       <c r="C153" s="2">
@@ -2518,10 +2517,10 @@
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A154" s="5" t="s">
+      <c r="A154" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="B154" s="5">
+      <c r="B154" s="1">
         <v>1</v>
       </c>
       <c r="C154" s="2">
@@ -2529,10 +2528,10 @@
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A155" s="5" t="s">
+      <c r="A155" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B155" s="5">
+      <c r="B155" s="1">
         <v>1</v>
       </c>
       <c r="C155" s="2">
@@ -2540,10 +2539,10 @@
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A156" s="5" t="s">
+      <c r="A156" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B156" s="5">
+      <c r="B156" s="1">
         <v>1</v>
       </c>
       <c r="C156" s="2">
@@ -2551,10 +2550,10 @@
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A157" s="5" t="s">
+      <c r="A157" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B157" s="5">
+      <c r="B157" s="1">
         <v>1</v>
       </c>
       <c r="C157" s="2">
@@ -2570,10 +2569,10 @@
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A159" s="5" t="s">
+      <c r="A159" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B159" s="5">
+      <c r="B159" s="1">
         <v>1</v>
       </c>
       <c r="C159" s="2">
@@ -2581,10 +2580,10 @@
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A160" s="5" t="s">
+      <c r="A160" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B160" s="5">
+      <c r="B160" s="1">
         <v>1</v>
       </c>
       <c r="C160" s="2">
@@ -2608,10 +2607,10 @@
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A163" s="5" t="s">
+      <c r="A163" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B163" s="5">
+      <c r="B163" s="1">
         <v>1</v>
       </c>
       <c r="C163" s="2">
@@ -2630,10 +2629,10 @@
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A165" s="5" t="s">
+      <c r="A165" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B165" s="5">
+      <c r="B165" s="1">
         <v>1</v>
       </c>
       <c r="C165" s="2">
@@ -2673,10 +2672,10 @@
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A170" s="5" t="s">
+      <c r="A170" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B170" s="5">
+      <c r="B170" s="1">
         <v>1</v>
       </c>
       <c r="C170" s="2">
@@ -2684,10 +2683,10 @@
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A171" s="5" t="s">
+      <c r="A171" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="B171" s="5">
+      <c r="B171" s="1">
         <v>1</v>
       </c>
       <c r="C171" s="2">
@@ -2719,10 +2718,10 @@
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A175" s="5" t="s">
+      <c r="A175" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="B175" s="5">
+      <c r="B175" s="1">
         <v>1</v>
       </c>
       <c r="C175" s="2">
@@ -2754,10 +2753,10 @@
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A179" s="5" t="s">
+      <c r="A179" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="B179" s="5">
+      <c r="B179" s="1">
         <v>1</v>
       </c>
       <c r="C179" s="2">
@@ -2773,10 +2772,10 @@
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A181" s="5" t="s">
+      <c r="A181" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B181" s="5">
+      <c r="B181" s="1">
         <v>1</v>
       </c>
       <c r="C181" s="2">
@@ -2784,10 +2783,10 @@
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A182" s="5" t="s">
+      <c r="A182" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B182" s="5">
+      <c r="B182" s="1">
         <v>1</v>
       </c>
       <c r="C182" s="2">
@@ -2833,10 +2832,10 @@
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A187" s="5" t="s">
+      <c r="A187" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B187" s="5">
+      <c r="B187" s="1">
         <v>1</v>
       </c>
       <c r="C187" s="2">
@@ -2844,10 +2843,10 @@
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A188" s="5" t="s">
+      <c r="A188" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B188" s="5">
+      <c r="B188" s="1">
         <v>1</v>
       </c>
       <c r="C188" s="2">
@@ -2879,10 +2878,10 @@
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A192" s="5" t="s">
+      <c r="A192" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="B192" s="5">
+      <c r="B192" s="1">
         <v>1</v>
       </c>
       <c r="C192" s="2">
@@ -2890,10 +2889,10 @@
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A193" s="5" t="s">
+      <c r="A193" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B193" s="5">
+      <c r="B193" s="1">
         <v>1</v>
       </c>
       <c r="C193" s="2">
@@ -2909,10 +2908,10 @@
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A195" s="5" t="s">
+      <c r="A195" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="B195" s="5">
+      <c r="B195" s="1">
         <v>1</v>
       </c>
       <c r="C195" s="2">
@@ -2944,10 +2943,10 @@
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A199" s="5" t="s">
+      <c r="A199" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="B199" s="5">
+      <c r="B199" s="1">
         <v>1</v>
       </c>
       <c r="C199" s="2">

</xml_diff>